<commit_message>
fix(quiz): refine question text and multi-column options for 120th exam problem #7 (#67, #82)
</commit_message>
<xml_diff>
--- a/excels/1급_기출문제_필기.xlsx
+++ b/excels/1급_기출문제_필기.xlsx
@@ -1,21 +1,20 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
-  <sheets>
-    <sheet name="문제" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="정답및해설" sheetId="2" state="visible" r:id="rId2"/>
-  </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties">
+  <Application>Microsoft Excel Compatible / Openpyxl 3.1.5</Application>
+  <AppVersion>3.1</AppVersion>
+</Properties>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <dc:creator>openpyxl</dc:creator>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-08-25T09:16:06Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-08-25T09:16:06Z</dcterms:modified>
+</cp:coreProperties>
+</file>
+
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
   <fonts count="1">
@@ -125,7 +124,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -408,7 +407,23 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
+  <sheets>
+    <sheet name="문제" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="정답및해설" sheetId="2" state="visible" r:id="rId2"/>
+  </sheets>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3197,38 +3212,38 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="n">
-        <v>67</v>
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>[제120회 기출 #7] 다음의 자료를 바탕으로 상품매출원가를 계산하여 결산분개한 것으로 옳은 것은?
+          <t>[제120회 기출 #7] 다음의 자료를 바탕으로 상품매출원가를 계산하여 결산분개할 때 차변과 대변에 올바른 것은?
 가. 기초상품재고액 1,100,000원
 나. 당기총상품매입액 4,550,000원
 다. 기말상품재고액 2,300,000원
-라. 당기총매출액 7,200,000원
-차변
-대변</t>
+라. 당기총매출액 7,200,000원</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>상품매출원가 3,350,000원</t>
+          <t>(차) 상품매출원가 3,350,000원  /  (대) 상품 3,350,000원</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>상품 3,850,000원</t>
+          <t>(차) 상품매출원가 3,850,000원  /  (대) 상품 3,850,000원</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>상품 3,350,000원</t>
+          <t>(차) 상품 3,350,000원  /  (대) 상품매출원가 3,350,000원</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>상품매출원가 3,850,000원</t>
+          <t>(차) 상품 3,850,000원  /  (대) 상품매출원가 3,850,000원</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -3842,38 +3857,38 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" t="n">
-        <v>82</v>
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>[제120회 B형 기출 #7] 다음의 자료를 바탕으로 상품매출원가를 계산하여 결산분개한 것으로 옳은 것은?
+          <t>[제120회 B형 기출 #7] 다음의 자료를 바탕으로 상품매출원가를 계산하여 결산분개할 때 차변과 대변에 올바른 것은?
 가. 기초상품재고액 1,100,000원
 나. 당기총상품매입액 4,550,000원
 다. 기말상품재고액 2,300,000원
-라. 당기총매출액 7,200,000원
-차변
-대변</t>
+라. 당기총매출액 7,200,000원</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>상품매출원가 3,350,000원</t>
+          <t>(차) 상품매출원가 3,350,000원  /  (대) 상품 3,350,000원</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>상품 3,850,000원</t>
+          <t>(차) 상품매출원가 3,850,000원  /  (대) 상품 3,850,000원</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>상품 3,350,000원</t>
+          <t>(차) 상품 3,350,000원  /  (대) 상품매출원가 3,350,000원</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>상품매출원가 3,850,000원</t>
+          <t>(차) 상품 3,850,000원  /  (대) 상품매출원가 3,850,000원</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -13056,7 +13071,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>